<commit_message>
Renommage du profil FRActProcedureDocument (#112) 20f3d6116cd73e255f022cbd12f1b6d170d85e27
</commit_message>
<xml_diff>
--- a/fixbugversion/ig/FRActSubstitutionLMCDAFHIR.xlsx
+++ b/fixbugversion/ig/FRActSubstitutionLMCDAFHIR.xlsx
@@ -31,7 +31,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0-snapshot</t>
+    <t>0.1.0-snapsnot</t>
   </si>
   <si>
     <t>Name</t>
@@ -55,7 +55,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-15T13:14:55+00:00</t>
+    <t>2026-04-15T14:22:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>